<commit_message>
Add downside rule: review gate when a scenario NPV is negative
</commit_message>
<xml_diff>
--- a/templates/business_case.xlsx
+++ b/templates/business_case.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -639,10 +639,17 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>- A negative scenario is a decision input, not a footnote. If the 3-year NPV is negative in any scenario, the case can only be approved with conditions: a review gate 3 months after go-live, and stop or rework if adoption or time saved fall to their pessimistic values.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Nothing in this workbook is protected. Results are recalculated when the file is opened.</t>
         </is>

</xml_diff>